<commit_message>
SQL listo para desactivar 22 fichas pobres que ya existen
Un solo script con candados (el SKU bueno tiene que estar activo y
con ese EAN). No suma stock salvo Cintapore. Excel: hoja de lo que
sí falta comprar y lo que solo necesita código de barras.

Co-authored-by: ibarraivane <ibarraivane@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pricing/reportes/duplicados_sin_barcode_20260914.xlsx
+++ b/pricing/reportes/duplicados_sin_barcode_20260914.xlsx
@@ -8,12 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="DESACTIVAR_ya_existen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="UNICOS_falta_EAN" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="NO_ESTAN_COMPRAR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DESACTIVAR_ya_existen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="UNICOS_falta_EAN" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DESACTIVAR_ya_existen'!$A$1:$J$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'UNICOS_falta_EAN'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NO_ESTAN_COMPRAR'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DESACTIVAR_ya_existen'!$A$1:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'UNICOS_falta_EAN'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +42,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -91,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -101,7 +108,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -469,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="64" customWidth="1" min="1" max="1"/>
@@ -520,30 +529,40 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Duplicados confirmados (desactivar el sin EAN)</t>
+          <t>Duplicados confirmados (SQL desactiva el sin EAN)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sin EAN pero únicos (solo falta código)</t>
+          <t>Sin EAN pero únicos (no desactivar)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>A comprar — no están en catálogo</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Único caso para pasar stock</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Cintapore FMX-301136 → FC-84500546 (el de EAN tiene 0)</t>
         </is>
@@ -564,7 +583,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Pedir</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Qué comprar (genérico)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Para qué</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Metformina 1000 mg 30 tabletas</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Diabetes — hoy solo hay 500 y 850</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Metformina 750 mg LP 30 tabletas</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Diabetes liberación prolongada</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Racecadotrilo 30 mg 18 sobres</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Diarrea niños — no hay Hidrasec ni genérico</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Racecadotrilo 10 mg 18 sobres</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Diarrea bebés</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Racecadotrilo 100 mg 9 cápsulas</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Diarrea adulto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Atenolol 50 mg 28 tabletas</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Presión — no hay betabloqueador</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Atenolol 100 mg 28 tabletas</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Presión</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -632,1122 +793,1074 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>FC-A0D320D1</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Amoxicilina 500 mg 12 cápsulas</t>
         </is>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>FC-49021570</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Amoxicilina 500 mg Caja con 12 cápsulas AMSA</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>7501349021570</t>
         </is>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>Misma caja AMSA. La ficha pobre es solo el genérico.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>FC-022543CD</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Valclan 500/125 mg 10 tabletas</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>FC-01007199</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>Valclan 500 mg / 125 mg Caja con 10 tabletas Wandel</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>7503001007199</t>
         </is>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Misma presentación 500/125. No confundir con Valclan 875.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>FC-7D1D9857</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Acetilsalicilico 100 mg 30 tabletas</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>FC-42803524</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Ácido acetilsalicílico 100 mg Caja con 30 tabletas beadvance</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>7501342803524</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Es AAS 100 mg, no Aspirina 500. El EAN de Aspirina ya se le había quitado.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>FC-95779436</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Ácido acetilsalicílico efervescente 300 mg C/20</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>EQ-ALP0300</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Acido Acetilsalicilico Ef 20 Tab 300 Mg</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>7501384504908</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>Misma caja Psicofarma 300 mg × 20.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>FC-B25B4654</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Cina (Ciprofloxacino) 750 mg 7 tabletas</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>FC-52200809</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Cina 750 mg Caja con 7 tabletas Landsteiner</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>7502225092486</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Cina es levofloxacino; la ficha pobre puso ciprofloxacino.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>FC-6C2878CF</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Budenova budesonida 0.125 mg/ml 5 amp × 2 ml</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="D7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>EQ-NOV165</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Budenova Susp .125 Mg/Ml 5 Amp 2ml</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>7501075726251</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="H7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>Misma Budenova Novag.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>FC-26EA40A4</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Raamcinet cetirizina 10 mg C/10</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>FC-27872123</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Raamcinet cetirizina 10 mg</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>7502227872123</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Misma caja C/10. Stocks 6 y 4: probable doble conteo.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>FC-44B6751A</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>LAÜR Adulto solución inyectable C/3</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="D9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>EQ-SON264</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Laur Solución Inyectable</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>7502001166981</t>
         </is>
       </c>
-      <c r="H9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="H9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>Adulto. El infantil (7502001167001) es otro SKU.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>FC-1321B34F</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Hidroxin hidroxizina 10 mg C/30</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>EQ-MAI099</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Hidroxin</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>785120754681</t>
         </is>
       </c>
-      <c r="H10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Misma Hidroxin Mavi 10 mg C/30.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>FC-AA7B0686</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Drosequim Adulto jarabe 300/160 mg 200 ml</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="D11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>EQ-QUM070</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Drosequim Ad 1 Jbe 300/160/200 Ml</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>7502223111400</t>
         </is>
       </c>
-      <c r="H11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="H11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>Mismo jarabe adulto Quimpharma.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>FC-926099D3</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Merthiolate Rojo Kohn 20 ml</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>FC-46601138</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Merthiolate Rojo Kohn 20 ml</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>7506346601138</t>
         </is>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Mismo nombre. Stocks 5 y 5: probable doble conteo.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>EQ-MAV401</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Dexpantenol 1 Cma 5% 30 G</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>FC-09749421</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Dexpantenol crema 5% 30 g (Maver Tattoo)</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>7502009749421</t>
         </is>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>Misma crema Maver 5% 30 g. Pamedan es otra marca.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>EQ-BRL072-1</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Lo Bruquin 2 Tab 150/200 Mg</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>EQ-BRL072</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Lo Bruquin Quinfamida, Albendazol</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>7502208894915</t>
         </is>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>SKU -1 sin EAN. Ambos con stock 10: el mismo lote contado dos veces.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>FMX-501619</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Eucalin-Miel Jarabe C/120 Ml</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="D15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>FC-08100013</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Eucalín jarabe miel y propóleo 120 ml</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>714908100013</t>
         </is>
       </c>
-      <c r="H15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="H15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>Carga Farma MX vs ficha completa.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>FMX-502465</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Colageno-Naturex Tabletas C/60</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="D16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>FC-9741524</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Naturex colágeno hidrolizado tabletas C/60</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>7502009741524</t>
         </is>
       </c>
-      <c r="H16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="H16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Carga Farma MX vs ficha Naturex.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>FMX-301136</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Cintapore cinta microporosa piel 2.5 cm x 5 m</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>FC-84500546</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Cintapore cinta microporosa piel 2.5 cm x 5m</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>7506484500546</t>
         </is>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="H17" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="9" t="inlineStr">
         <is>
           <t>SÍ — el de EAN tiene 0</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>El de EAN tiene stock 0: pasar las 2 piezas a ese SKU.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>FMX-501000</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Gelcavit-Colors Capsulas C/30</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="D18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>FC-30713547</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Gelcavit Colors capsulas 0.62 g C/30</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>7501130713547</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="H18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Misma variante Colors.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>FMX-500998</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Gelcavit-Platinum Capsulas C/30</t>
         </is>
       </c>
-      <c r="D19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="D19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>FC-30713851</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Gelcavit Platinum capsulas 1.39 g C/30</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>7501130713851</t>
         </is>
       </c>
-      <c r="H19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="H19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>Misma variante Platinum.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>FMX-501003</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Gelcavit-Q-10 Capsulas C/30</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="D20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>FC-13071164</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Gelcavit Q-10 coenzima Q10 jalea real C/30</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>7501130711642</t>
         </is>
       </c>
-      <c r="H20" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="H20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>Misma variante Q-10.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>FMX-505937</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Pleniform-40 Tabletas C/30</t>
         </is>
       </c>
-      <c r="D21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="D21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>FC-1041884</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Biomiral Pleniform 40 isoflavonas soya C/30</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>7503181041884</t>
         </is>
       </c>
-      <c r="H21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="H21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J21" s="8" t="inlineStr">
         <is>
           <t>Mismo Pleniform 40.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>FMX-302947</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Citrato Magnesio/Lecitina Soya-Naturex Capsulas C/30</t>
         </is>
       </c>
-      <c r="D22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="D22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>FC-9892403</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Naturex citrato de magnesio y lecitina de soya C/30</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>7502259892403</t>
         </is>
       </c>
-      <c r="H22" s="5" t="n">
+      <c r="H22" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Misma Naturex citrato + lecitina.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Desactivar ficha pobre</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>FMX-506935</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Normogotero-Sensimedical Piezas C/1 S/Aguja</t>
         </is>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>FC-22322395</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Normogotero Sensi Medical</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>7506022322395</t>
         </is>
       </c>
-      <c r="H23" s="6" t="n">
+      <c r="H23" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>NO — no sumar (posible doble conteo)</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="J23" s="8" t="inlineStr">
         <is>
           <t>Mismo gotero. Stocks 5 y 5: probable doble conteo.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Desactivar ficha pobre</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>FC-89F00320</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Mercurio Arnica C/25</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>FC-00003920</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Arnica Mercurio</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>3311000003944</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>NO — no sumar (posible doble conteo)</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>Árnica Mercurio en glóbulos C/25.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J24"/>
+  <autoFilter ref="A1:J23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1779,362 +1892,602 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>FC-DB4A39AE</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Eferox (Cefalexina) 500 mg 12 comprimidos</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>No hay otra Eferox. Solo falta EAN.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>FC-63975795</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Gentamicina 1 mg 25 comprimidos</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>No es la gentamicina inyectable 160 mg AMSA.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>FC-262F2A30</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Irbesartan 150 mg 14 tabletas AMSA</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Los LGEN son 28 tabletas; AMSA 300 mg es otra dosis.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>FC-2E5B7248</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Reumatol 60 g</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Único. Sin pareja con EAN.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>FC-3E863E37</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Tratidri gel 500/50 mg 60 g</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Único.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>FC-405A75E3</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Ursodesoxicolico 250 mg 50 cápsulas</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="C7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Único.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>EQ-SON225</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Norkin 7 Caps 40 Mg</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Único.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>EQ-AMS234</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Pregabalina 150 mg C/28 cápsulas AMSA</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="C9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Hay 75 mg con EAN; esta dosis 150 no.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>FC-C22EBFE6</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Perilla N2</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Tamaño distinto a la N1 (sí tiene EAN).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>FC-614E4F82</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Perilla N3</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>Tamaño distinto a la N1.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>FC-FFC25DD1</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Perilla N4</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Tamaño distinto a la N1.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>FC-A871D831</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Perilla N6</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Tamaño distinto a la N1.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>FC-9A1C64E7</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Perilla Edigar N O Caja</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Revisar si es caja o pieza; no es la N1.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>FC-C8B741F6</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>FC producto botiquín</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Ficha vacía. Identificar qué pieza es.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>FMX-301721</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Vita/Kid/C Jarabe C/240 Ml</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Único.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>FMX-302884</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Sol-Sun Crema C/50 Gr 50-Fps</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Único.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>FMX-502700</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>La-Femme Capsulas C/30</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Único.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>FMX-301138</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Cinta-Microporosa-Codifarma 2.5 cm × 5 m blanco</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Otra marca (Codifarma), no Cintapore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>FC-IFC-83368</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Gel sanitizante Dibar 50 ml</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>FC-IFC-83613</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Venditas adhesivas redondas Jayor C/100</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>FC-IFC-83490</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Guantes de nitrilo azul chico C/100</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>FC-IFC-83125</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Guantes de nitrilo azul grande C/100</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>FC-IFC-83947</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Guantes de nitrilo negro mediano C/100</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>FC-IFC-82084</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Brocha para tinte con peine de cola</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>FC-IFC-83552</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Venda Stick cohesiva 2 pulg × 4.5 m rojo</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>FC-IFC-82912A</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Venda Stick cohesiva 3 pulg × 4.5 m azul</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>FC-IFC-82912P</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Venda Stick cohesiva 3 pulg × 4.5 m piel</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>FC-EXP-PALM8</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Palmolive Neutro Balance jabón 100 g 8 pack</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Único. Falta EAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>FC-89F00320</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Mercurio Arnica C/25</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Parece Árnica Mercurio glóbulos, pero no lo desactivo sin ver la caja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>FC-DFF99C3F</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Mercurio (ficha mezclada)</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>La ficha está sucia (árnica + jarabe de granada). Identificar en anaquel.</t>
         </is>
       </c>
     </row>

</xml_diff>